<commit_message>
v6 Fig.6: markers on every 20-min point; Fig.7 redrawn to show candidate narrowing (raw per-judgment timeline + per-round learning curves, FIO/Varmail 45->5)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figs/data/fig6_v6_mixT.xlsx
+++ b/figs/data/fig6_v6_mixT.xlsx
@@ -178,9 +178,16 @@
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="none"/>
+            <symbol val="circle"/>
+            <size val="4"/>
             <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="E3A33B"/>
+              </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:solidFill>
+                  <a:srgbClr val="E3A33B"/>
+                </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -214,9 +221,16 @@
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="none"/>
+            <symbol val="circle"/>
+            <size val="4"/>
             <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="9A9994"/>
+              </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:solidFill>
+                  <a:srgbClr val="9A9994"/>
+                </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -250,9 +264,16 @@
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="none"/>
+            <symbol val="circle"/>
+            <size val="4"/>
             <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="2B2A28"/>
+              </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:solidFill>
+                  <a:srgbClr val="2B2A28"/>
+                </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -286,9 +307,16 @@
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="none"/>
+            <symbol val="circle"/>
+            <size val="6"/>
             <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:solidFill>
+                  <a:srgbClr val="2A78D6"/>
+                </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -2772,7 +2800,7 @@
     <row r="33">
       <c r="J33" t="inlineStr">
         <is>
-          <t>점선 = 워크로드 전환, 위 글자 = 그 구간의 워크로드. CAT-37·50은 DB 300k 레코드(나머지는 250k). 정책마다 1회 실행. v6·CAT-37·50 = 두 번째 PC, CAT-47 = 이 PC.</t>
+          <t>점 = 20분 구간 1개. 점선 = 워크로드 전환, 위 글자 = 그 구간의 워크로드. CAT-37·50은 DB 300k 레코드(나머지는 250k). 정책마다 1회 실행. v6·CAT-37·50 = 두 번째 PC, CAT-47 = 이 PC.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel charts: back to the construction of the earlier working figures (named line series in the legend); no data-label helper series, no hidden legend entries, no image sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figs/data/fig6_v6_mixT.xlsx
+++ b/figs/data/fig6_v6_mixT.xlsx
@@ -621,357 +621,6 @@
           </yVal>
           <smooth val="0"/>
         </ser>
-        <ser>
-          <idx val="12"/>
-          <order val="12"/>
-          <tx>
-            <strRef>
-              <f>'그림6 WAF 추이'!AA1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <dLbls>
-            <dLblPos val="t"/>
-            <showLegendKey val="0"/>
-            <showVal val="0"/>
-            <showSerName val="1"/>
-          </dLbls>
-          <xVal>
-            <numRef>
-              <f>'그림6 WAF 추이'!$Z$2</f>
-            </numRef>
-          </xVal>
-          <yVal>
-            <numRef>
-              <f>'그림6 WAF 추이'!$AA$2</f>
-            </numRef>
-          </yVal>
-        </ser>
-        <ser>
-          <idx val="13"/>
-          <order val="13"/>
-          <tx>
-            <strRef>
-              <f>'그림6 WAF 추이'!AC1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <dLbls>
-            <dLblPos val="t"/>
-            <showLegendKey val="0"/>
-            <showVal val="0"/>
-            <showSerName val="1"/>
-          </dLbls>
-          <xVal>
-            <numRef>
-              <f>'그림6 WAF 추이'!$AB$2</f>
-            </numRef>
-          </xVal>
-          <yVal>
-            <numRef>
-              <f>'그림6 WAF 추이'!$AC$2</f>
-            </numRef>
-          </yVal>
-        </ser>
-        <ser>
-          <idx val="14"/>
-          <order val="14"/>
-          <tx>
-            <strRef>
-              <f>'그림6 WAF 추이'!AE1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <dLbls>
-            <dLblPos val="t"/>
-            <showLegendKey val="0"/>
-            <showVal val="0"/>
-            <showSerName val="1"/>
-          </dLbls>
-          <xVal>
-            <numRef>
-              <f>'그림6 WAF 추이'!$AD$2</f>
-            </numRef>
-          </xVal>
-          <yVal>
-            <numRef>
-              <f>'그림6 WAF 추이'!$AE$2</f>
-            </numRef>
-          </yVal>
-        </ser>
-        <ser>
-          <idx val="15"/>
-          <order val="15"/>
-          <tx>
-            <strRef>
-              <f>'그림6 WAF 추이'!AG1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <dLbls>
-            <dLblPos val="t"/>
-            <showLegendKey val="0"/>
-            <showVal val="0"/>
-            <showSerName val="1"/>
-          </dLbls>
-          <xVal>
-            <numRef>
-              <f>'그림6 WAF 추이'!$AF$2</f>
-            </numRef>
-          </xVal>
-          <yVal>
-            <numRef>
-              <f>'그림6 WAF 추이'!$AG$2</f>
-            </numRef>
-          </yVal>
-        </ser>
-        <ser>
-          <idx val="16"/>
-          <order val="16"/>
-          <tx>
-            <strRef>
-              <f>'그림6 WAF 추이'!AI1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <dLbls>
-            <dLblPos val="t"/>
-            <showLegendKey val="0"/>
-            <showVal val="0"/>
-            <showSerName val="1"/>
-          </dLbls>
-          <xVal>
-            <numRef>
-              <f>'그림6 WAF 추이'!$AH$2</f>
-            </numRef>
-          </xVal>
-          <yVal>
-            <numRef>
-              <f>'그림6 WAF 추이'!$AI$2</f>
-            </numRef>
-          </yVal>
-        </ser>
-        <ser>
-          <idx val="17"/>
-          <order val="17"/>
-          <tx>
-            <strRef>
-              <f>'그림6 WAF 추이'!AK1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <dLbls>
-            <dLblPos val="t"/>
-            <showLegendKey val="0"/>
-            <showVal val="0"/>
-            <showSerName val="1"/>
-          </dLbls>
-          <xVal>
-            <numRef>
-              <f>'그림6 WAF 추이'!$AJ$2</f>
-            </numRef>
-          </xVal>
-          <yVal>
-            <numRef>
-              <f>'그림6 WAF 추이'!$AK$2</f>
-            </numRef>
-          </yVal>
-        </ser>
-        <ser>
-          <idx val="18"/>
-          <order val="18"/>
-          <tx>
-            <strRef>
-              <f>'그림6 WAF 추이'!AM1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <dLbls>
-            <dLblPos val="t"/>
-            <showLegendKey val="0"/>
-            <showVal val="0"/>
-            <showSerName val="1"/>
-          </dLbls>
-          <xVal>
-            <numRef>
-              <f>'그림6 WAF 추이'!$AL$2</f>
-            </numRef>
-          </xVal>
-          <yVal>
-            <numRef>
-              <f>'그림6 WAF 추이'!$AM$2</f>
-            </numRef>
-          </yVal>
-        </ser>
-        <ser>
-          <idx val="19"/>
-          <order val="19"/>
-          <tx>
-            <strRef>
-              <f>'그림6 WAF 추이'!AO1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <dLbls>
-            <dLblPos val="t"/>
-            <showLegendKey val="0"/>
-            <showVal val="0"/>
-            <showSerName val="1"/>
-          </dLbls>
-          <xVal>
-            <numRef>
-              <f>'그림6 WAF 추이'!$AN$2</f>
-            </numRef>
-          </xVal>
-          <yVal>
-            <numRef>
-              <f>'그림6 WAF 추이'!$AO$2</f>
-            </numRef>
-          </yVal>
-        </ser>
-        <ser>
-          <idx val="20"/>
-          <order val="20"/>
-          <tx>
-            <strRef>
-              <f>'그림6 WAF 추이'!AQ1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <dLbls>
-            <dLblPos val="t"/>
-            <showLegendKey val="0"/>
-            <showVal val="0"/>
-            <showSerName val="1"/>
-          </dLbls>
-          <xVal>
-            <numRef>
-              <f>'그림6 WAF 추이'!$AP$2</f>
-            </numRef>
-          </xVal>
-          <yVal>
-            <numRef>
-              <f>'그림6 WAF 추이'!$AQ$2</f>
-            </numRef>
-          </yVal>
-        </ser>
         <axId val="10"/>
         <axId val="20"/>
       </scatterChart>
@@ -1036,74 +685,6 @@
     </plotArea>
     <legend>
       <legendPos val="b"/>
-      <legendEntry>
-        <idx val="4"/>
-        <delete val="1"/>
-      </legendEntry>
-      <legendEntry>
-        <idx val="5"/>
-        <delete val="1"/>
-      </legendEntry>
-      <legendEntry>
-        <idx val="6"/>
-        <delete val="1"/>
-      </legendEntry>
-      <legendEntry>
-        <idx val="7"/>
-        <delete val="1"/>
-      </legendEntry>
-      <legendEntry>
-        <idx val="8"/>
-        <delete val="1"/>
-      </legendEntry>
-      <legendEntry>
-        <idx val="9"/>
-        <delete val="1"/>
-      </legendEntry>
-      <legendEntry>
-        <idx val="10"/>
-        <delete val="1"/>
-      </legendEntry>
-      <legendEntry>
-        <idx val="11"/>
-        <delete val="1"/>
-      </legendEntry>
-      <legendEntry>
-        <idx val="12"/>
-        <delete val="1"/>
-      </legendEntry>
-      <legendEntry>
-        <idx val="13"/>
-        <delete val="1"/>
-      </legendEntry>
-      <legendEntry>
-        <idx val="14"/>
-        <delete val="1"/>
-      </legendEntry>
-      <legendEntry>
-        <idx val="15"/>
-        <delete val="1"/>
-      </legendEntry>
-      <legendEntry>
-        <idx val="16"/>
-        <delete val="1"/>
-      </legendEntry>
-      <legendEntry>
-        <idx val="17"/>
-        <delete val="1"/>
-      </legendEntry>
-      <legendEntry>
-        <idx val="18"/>
-        <delete val="1"/>
-      </legendEntry>
-      <legendEntry>
-        <idx val="19"/>
-        <delete val="1"/>
-      </legendEntry>
-      <legendEntry>
-        <idx val="20"/>
-        <delete val="1"/>
-      </legendEntry>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -1698,82 +1279,82 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>전환1 시간</t>
+          <t>→ 2.OLTP 시간</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>전환1</t>
+          <t>→ 2.OLTP</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>전환2 시간</t>
+          <t>→ 3.Varmail 시간</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>전환2</t>
+          <t>→ 3.Varmail</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>전환3 시간</t>
+          <t>→ 4.YCSB-A 시간</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>전환3</t>
+          <t>→ 4.YCSB-A</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>전환4 시간</t>
+          <t>→ 5.YCSB-B 시간</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>전환4</t>
+          <t>→ 5.YCSB-B</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>전환5 시간</t>
+          <t>→ 6.FIO-Fast 시간</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>전환5</t>
+          <t>→ 6.FIO-Fast</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>전환6 시간</t>
+          <t>→ 7.Varmail 시간</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>전환6</t>
+          <t>→ 7.Varmail</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>전환7 시간</t>
+          <t>→ 8.YCSB-A 시간</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>전환7</t>
+          <t>→ 8.YCSB-A</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>전환8 시간</t>
+          <t>→ 9.OLTP 시간</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>전환8</t>
+          <t>→ 9.OLTP</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
fig6/fig7 (v6 mixT) xlsx: dark paper colors, all chart lines and borders 2 pt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figs/data/fig6_v6_mixT.xlsx
+++ b/figs/data/fig6_v6_mixT.xlsx
@@ -170,9 +170,9 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
               <a:solidFill>
-                <a:srgbClr val="E3A33B"/>
+                <a:srgbClr val="8B2E16"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -182,11 +182,11 @@
             <size val="4"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="E3A33B"/>
+                <a:srgbClr val="8B2E16"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:solidFill>
-                  <a:srgbClr val="E3A33B"/>
+                  <a:srgbClr val="8B2E16"/>
                 </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -213,9 +213,9 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
               <a:solidFill>
-                <a:srgbClr val="9A9994"/>
+                <a:srgbClr val="5A5A5A"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -225,11 +225,11 @@
             <size val="4"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="9A9994"/>
+                <a:srgbClr val="5A5A5A"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:solidFill>
-                  <a:srgbClr val="9A9994"/>
+                  <a:srgbClr val="5A5A5A"/>
                 </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -256,9 +256,9 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
               <a:solidFill>
-                <a:srgbClr val="2B2A28"/>
+                <a:srgbClr val="1A1A1A"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -268,11 +268,11 @@
             <size val="4"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="2B2A28"/>
+                <a:srgbClr val="1A1A1A"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:solidFill>
-                  <a:srgbClr val="2B2A28"/>
+                  <a:srgbClr val="1A1A1A"/>
                 </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -299,9 +299,9 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="34925">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
               <a:solidFill>
-                <a:srgbClr val="2A78D6"/>
+                <a:srgbClr val="0B3C8C"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -311,11 +311,11 @@
             <size val="6"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="2A78D6"/>
+                <a:srgbClr val="0B3C8C"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:solidFill>
-                  <a:srgbClr val="2A78D6"/>
+                  <a:srgbClr val="0B3C8C"/>
                 </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -342,9 +342,9 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
               <a:solidFill>
-                <a:srgbClr val="8A8984"/>
+                <a:srgbClr val="404040"/>
               </a:solidFill>
               <a:prstDash val="dash"/>
             </a:ln>
@@ -378,9 +378,9 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
               <a:solidFill>
-                <a:srgbClr val="8A8984"/>
+                <a:srgbClr val="404040"/>
               </a:solidFill>
               <a:prstDash val="dash"/>
             </a:ln>
@@ -414,9 +414,9 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
               <a:solidFill>
-                <a:srgbClr val="8A8984"/>
+                <a:srgbClr val="404040"/>
               </a:solidFill>
               <a:prstDash val="dash"/>
             </a:ln>
@@ -450,9 +450,9 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
               <a:solidFill>
-                <a:srgbClr val="8A8984"/>
+                <a:srgbClr val="404040"/>
               </a:solidFill>
               <a:prstDash val="dash"/>
             </a:ln>
@@ -486,9 +486,9 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
               <a:solidFill>
-                <a:srgbClr val="8A8984"/>
+                <a:srgbClr val="404040"/>
               </a:solidFill>
               <a:prstDash val="dash"/>
             </a:ln>
@@ -522,9 +522,9 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
               <a:solidFill>
-                <a:srgbClr val="8A8984"/>
+                <a:srgbClr val="404040"/>
               </a:solidFill>
               <a:prstDash val="dash"/>
             </a:ln>
@@ -558,9 +558,9 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
               <a:solidFill>
-                <a:srgbClr val="8A8984"/>
+                <a:srgbClr val="404040"/>
               </a:solidFill>
               <a:prstDash val="dash"/>
             </a:ln>
@@ -594,9 +594,9 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
               <a:solidFill>
-                <a:srgbClr val="8A8984"/>
+                <a:srgbClr val="404040"/>
               </a:solidFill>
               <a:prstDash val="dash"/>
             </a:ln>
@@ -689,6 +689,14 @@
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
+  <spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
+      <a:solidFill>
+        <a:srgbClr val="1A1A1A"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </spPr>
 </chartSpace>
 </file>
 
@@ -724,10 +732,12 @@
           </tx>
           <spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="E3A33B"/>
+              <a:srgbClr val="8B2E16"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:noFill/>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -752,10 +762,12 @@
           </tx>
           <spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="9A9994"/>
+              <a:srgbClr val="5A5A5A"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:noFill/>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -780,10 +792,12 @@
           </tx>
           <spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="2B2A28"/>
+              <a:srgbClr val="1A1A1A"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:noFill/>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -808,10 +822,12 @@
           </tx>
           <spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="2A78D6"/>
+              <a:srgbClr val="0B3C8C"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:noFill/>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -877,6 +893,14 @@
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
+  <spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
+      <a:solidFill>
+        <a:srgbClr val="1A1A1A"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </spPr>
 </chartSpace>
 </file>
 

</xml_diff>